<commit_message>
updating timings based upon method inlining
</commit_message>
<xml_diff>
--- a/objeck-lang/wip/timming/times.xlsx
+++ b/objeck-lang/wip/timming/times.xlsx
@@ -168,7 +168,7 @@
                   <c:v>0.90075</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8684915</c:v>
+                  <c:v>0.478394</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.38547825</c:v>
@@ -177,24 +177,24 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="546246792"/>
-        <c:axId val="546238712"/>
+        <c:axId val="565214840"/>
+        <c:axId val="565203480"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="546246792"/>
+        <c:axId val="565214840"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="546238712"/>
+        <c:crossAx val="565203480"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="546238712"/>
+        <c:axId val="565203480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -202,7 +202,7 @@
         <c:majorGridlines/>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="546246792"/>
+        <c:crossAx val="565214840"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -615,7 +615,7 @@
         <v>0.877</v>
       </c>
       <c r="C2">
-        <v>0.86802199999999996</v>
+        <v>0.47585300000000003</v>
       </c>
       <c r="D2">
         <v>0.38568599999999997</v>
@@ -629,7 +629,7 @@
         <v>0.88300000000000001</v>
       </c>
       <c r="C3">
-        <v>0.86253899999999994</v>
+        <v>0.48208499999999999</v>
       </c>
       <c r="D3">
         <v>0.38621100000000003</v>
@@ -643,7 +643,7 @@
         <v>0.93100000000000005</v>
       </c>
       <c r="C4">
-        <v>0.87425799999999998</v>
+        <v>0.47908600000000001</v>
       </c>
       <c r="D4">
         <v>0.38455899999999998</v>
@@ -657,7 +657,7 @@
         <v>0.91200000000000003</v>
       </c>
       <c r="C5">
-        <v>0.869147</v>
+        <v>0.47655199999999998</v>
       </c>
       <c r="D5">
         <v>0.38545699999999999</v>
@@ -674,7 +674,7 @@
       </c>
       <c r="C6">
         <f>AVERAGE(C2:C5)</f>
-        <v>0.86849149999999997</v>
+        <v>0.47839399999999999</v>
       </c>
       <c r="D6">
         <f>AVERAGE(D2:D5)</f>
@@ -684,10 +684,11 @@
     <row r="8" spans="1:4">
       <c r="A8">
         <f>ABS(C6/A6-1)</f>
-        <v>0.947658611478154</v>
+        <v>0.97116862258235115</v>
       </c>
     </row>
   </sheetData>
+  <sheetCalcPr fullCalcOnLoad="1"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>